<commit_message>
tested from nominal start proposal
</commit_message>
<xml_diff>
--- a/Probability_Estimates.xlsx
+++ b/Probability_Estimates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://office365stanford-my.sharepoint.com/personal/datsimp_stanford_edu/Documents/Stanford/AA228V/Final Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="147" documentId="11_F25DC773A252ABDACC10489BB95959C25ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{132B2799-20DB-4743-A498-69275D801A35}"/>
+  <xr:revisionPtr revIDLastSave="173" documentId="11_F25DC773A252ABDACC10489BB95959C25ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{284B7CAA-DCE0-4AFD-ACC9-CAF76465CD87}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="123">
   <si>
     <t>p_fail_est</t>
   </si>
@@ -351,28 +351,61 @@
     <t>Direct Estimation Results (Parallel Execution - 1000 Trials)</t>
   </si>
   <si>
-    <t>No Failure: 98.70% (987/1000)</t>
-  </si>
-  <si>
-    <t>Budget runs out (Total Cost): 1.20% (12/1000)</t>
-  </si>
-  <si>
     <t>Out of Time (Total Time): 0.00% (0/1000)</t>
   </si>
   <si>
-    <t>Drones got Stuck (Stuck Count): 0.10% (1/1000)</t>
-  </si>
-  <si>
     <t>Expert Direct Estimation</t>
   </si>
   <si>
-    <t>No Failure: 76.90% (769/1000)</t>
-  </si>
-  <si>
-    <t>Budget runs out (Total Cost): 21.20% (212/1000)</t>
-  </si>
-  <si>
-    <t>Drones got Stuck (Stuck Count): 1.90% (19/1000)</t>
+    <t>No Failure: 78.80% (788/1000)</t>
+  </si>
+  <si>
+    <t>Budget runs out (Total Cost): 19.70% (197/1000)</t>
+  </si>
+  <si>
+    <t>Drones got Stuck (Stuck Count): 1.50% (15/1000)</t>
+  </si>
+  <si>
+    <t>No Failure: 99.20% (992/1000)</t>
+  </si>
+  <si>
+    <t>Budget runs out (Total Cost): 0.80% (8/1000)</t>
+  </si>
+  <si>
+    <t>Drones got Stuck (Stuck Count): 0.00% (0/1000)</t>
+  </si>
+  <si>
+    <t>Nominal AIS</t>
+  </si>
+  <si>
+    <t>[0.93315893 0.55517258 0.46173623 0.07074068 0.0122179  0.79806457</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1.08129142]</t>
+  </si>
+  <si>
+    <t>[0.9330196  0.56749355 0.45196872 0.05772039 0.01157633 0.85691923</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1.66575544]</t>
+  </si>
+  <si>
+    <t>Estimated Probability of Failure (Nominal p): 6.105502e-02</t>
+  </si>
+  <si>
+    <t>Failure Rate of Proposal Distribution (Expert q): 84.00%</t>
+  </si>
+  <si>
+    <t>[0.96081279 0.30854117 0.55747985 0.03725574 0.01354655 0.87393467</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1.04344042]</t>
+  </si>
+  <si>
+    <t>Estimated Probability of Failure (Nominal p): 1.287776e-01</t>
+  </si>
+  <si>
+    <t>Failure Rate of Proposal Distribution (Expert q): 36.00%</t>
   </si>
 </sst>
 </file>
@@ -3598,87 +3631,197 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A171119-0B35-4C83-A844-A339EB12F364}">
-  <dimension ref="B2:B21"/>
+  <dimension ref="B2:H32"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="H2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B5" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="H5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B6" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="H6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B8" t="s">
+        <v>110</v>
+      </c>
+      <c r="H8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B9" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.4">
-      <c r="B8" t="s">
+      <c r="H9" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B10" t="s">
+        <v>111</v>
+      </c>
+      <c r="H10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H12" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.4">
-      <c r="B9" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.4">
-      <c r="B10" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.4">
-      <c r="B13" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B15" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="H15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B16" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="H16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B17" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="H17" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B18" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.4">
+        <v>106</v>
+      </c>
+      <c r="H18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B19" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+      <c r="H19" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B20" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.4">
+        <v>104</v>
+      </c>
+      <c r="H20" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B21" t="s">
-        <v>111</v>
+        <v>108</v>
+      </c>
+      <c r="H21" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H22" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H25" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H28" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H29" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H30" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H31" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="H32" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>